<commit_message>
feat(ai_eff): rename weighting in test files
</commit_message>
<xml_diff>
--- a/test_files/csv_test_files/COS10001-Tasks.xlsx
+++ b/test_files/csv_test_files/COS10001-Tasks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eliya/Dev/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/steven/repos/ontrack/doubtfire-deploy/doubtfire-api/test_files/csv_test_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849C7394-8847-1543-B8D9-CBCAA2832C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBD7C10D-0C9E-DF43-8EE7-7D4F3D712590}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="800" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="28800" windowHeight="17260" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="COS10001-Tasks" sheetId="1" r:id="rId1"/>
@@ -47,9 +47,6 @@
     <t>description</t>
   </si>
   <si>
-    <t>weighting</t>
-  </si>
-  <si>
     <t>target_grade</t>
   </si>
   <si>
@@ -138,6 +135,9 @@
   </si>
   <si>
     <t>discussion_prompts</t>
+  </si>
+  <si>
+    <t>estimated_hours</t>
   </si>
 </sst>
 </file>
@@ -371,6 +371,7 @@
   <dimension ref="A1:AA2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="20.5" customWidth="1"/>
     <col min="20" max="20" width="32" customWidth="1"/>
     <col min="21" max="21" width="24.33203125" customWidth="1"/>
@@ -392,87 +393,87 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
-        <v>22</v>
-      </c>
       <c r="X1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y1" t="s">
         <v>30</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>31</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>32</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
       </c>
       <c r="D2">
         <v>2</v>
@@ -495,28 +496,28 @@
         <v>50</v>
       </c>
       <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="L2" t="s">
         <v>26</v>
-      </c>
-      <c r="L2" t="s">
-        <v>27</v>
       </c>
       <c r="M2">
         <v>-1</v>
       </c>
       <c r="N2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="O2">
         <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q2">
         <v>13</v>
       </c>
       <c r="R2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Y2" t="b">
         <v>0</v>

</xml_diff>